<commit_message>
Update portfolio presentation and document signatures
</commit_message>
<xml_diff>
--- a/01-spreadsheet-cleanup.xlsx
+++ b/01-spreadsheet-cleanup.xlsx
@@ -290,9 +290,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Portfolio">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Portfolio">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -342,7 +342,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Portfolio">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>